<commit_message>
docs: relax properties for minor release
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.1.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anakonrad/Library/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0FB884F-CCDB-D643-A787-F700A1E15B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{935837CE-90B2-6C41-9184-09A5A911027E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4900" yWindow="-26760" windowWidth="42960" windowHeight="25280" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17380" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1876" uniqueCount="688">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1880" uniqueCount="688">
   <si>
     <t>Property label</t>
   </si>
@@ -1341,9 +1341,6 @@
     <t>https://publications.europa.eu/resource/authority/country</t>
   </si>
   <si>
-    <t>Use the appropriate term from the EU authority table. Example for the Netherlands: http://publications.europa.eu/resource/authority/country/NLD</t>
-  </si>
-  <si>
     <t>email</t>
   </si>
   <si>
@@ -1439,9 +1436,6 @@
     <t>healthdcatap:publishernote</t>
   </si>
   <si>
-    <t>This property can be repeated for parallel language versions of the publisher notes. Example: "Sciensano is a research institute and the national public health institute of Belgium. It is a so-called federal scientific institution that operates under the authority of the federal minister of Public Health and the federal minister of Agriculture of Belgium."@en</t>
-  </si>
-  <si>
     <t>publisher type</t>
   </si>
   <si>
@@ -1452,25 +1446,6 @@
   </si>
   <si>
     <t>https://raw.githubusercontent.com/SEMICeu/ADMS-AP/master/purl.org/ADMS_SKOS_v1.00.rdf</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Display"/>
-      </rPr>
-      <t>Current status</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Display"/>
-      </rPr>
-      <t>: Specifically for the health domain, a controlled vocabulary is being developed to include commonly recognised health publishers. This vocabulary is currently under development. Version 1.0 includes the following types: Academia-ScientificOrganisation, Company, IndustryConsortium, LocalAuthority, NationalAuthority, NonGovernmentalOrganisation, NonProfitOrganisation, PrivateIndividual, RegionalAuthority, StandardisationBody and SupraNationalAuthority. These should use the following URL: http://purl.org/adms/publishertype/[type].</t>
-    </r>
   </si>
   <si>
     <t>This property should be filled using ADMS vocabulary (http://purl.org/adms/publishertype/1.0)</t>
@@ -2625,54 +2600,155 @@
 If a limit is known, provide both dcat:startDate and dcat:endDate.</t>
   </si>
   <si>
-    <t>Indicate with this property in case the Distribution is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
+    <t>alternative</t>
+  </si>
+  <si>
+    <t>An alternative name for the dataset.</t>
+  </si>
+  <si>
+    <t>dct:alternative</t>
+  </si>
+  <si>
+    <t>This property contains an alternative name for the Dataset. This property can be repeated for parallel language versions of the alternative name.</t>
+  </si>
+  <si>
+    <t>landing page</t>
+  </si>
+  <si>
+    <t>A web page that provides access to the Dataset, its Distributions and/or additional information.</t>
+  </si>
+  <si>
+    <t>It is intended to point to a landing page at the original data provider, not to a page on a site of a third party, such as an aggregator.</t>
+  </si>
+  <si>
+    <t>provenance</t>
+  </si>
+  <si>
+    <t>A statement about the lineage of a Dataset.</t>
+  </si>
+  <si>
+    <t>Information about how the data was collected, including methodologies, tools, and protocols used, this property can be repeated for different versions of the provenance (e.g. the provenance in different languages).</t>
+  </si>
+  <si>
+    <t>dct:provenance</t>
+  </si>
+  <si>
+    <t>dct:ProvenanceStatement</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Note</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: This property will be deprecated in the next major release.
+Use the appropriate term from the EU authority table. Example for the Netherlands: http://publications.europa.eu/resource/authority/country/NLD</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>Note</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>: This property will be deprecated in the next major release.
+This property can be repeated for parallel language versions of the publisher notes. Example: "Sciensano is a research institute and the national public health institute of Belgium. It is a so-called federal scientific institution that operates under the authority of the federal minister of Public Health and the federal minister of Agriculture of Belgium."@en</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+      </rPr>
+      <t xml:space="preserve">Note: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+      </rPr>
+      <t>This property will be deprecated in the next major release.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+      </rPr>
+      <t xml:space="preserve">
+Current status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+      </rPr>
+      <t>: Specifically for the health domain, a controlled vocabulary is being developed to include commonly recognised health publishers. This vocabulary is currently under development. Version 1.0 includes the following types: Academia-ScientificOrganisation, Company, IndustryConsortium, LocalAuthority, NationalAuthority, NonGovernmentalOrganisation, NonProfitOrganisation, PrivateIndividual, RegionalAuthority, StandardisationBody and SupraNationalAuthority. These should use the following URL: http://purl.org/adms/publishertype/[type].</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>Note</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>: This property will be deprecated in the upcoming major release. 
+Indicate with this property in case the Distribution is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
 This property makes use of the class dct:PeriodOfTime, in which a start and end date can be provided.
 If the Distribution is available indefinitely, leave the property empty (cardinality is 0..1; it is only meaningful when a retention limit applies).
 If only a start is known, provide dcat:startDate only (open-ended interval, as allowed by dct:PeriodOfTime).
 If a limit is known, provide both dcat:startDate and dcat:endDate.</t>
-  </si>
-  <si>
-    <t>alternative</t>
-  </si>
-  <si>
-    <t>An alternative name for the dataset.</t>
-  </si>
-  <si>
-    <t>dct:alternative</t>
-  </si>
-  <si>
-    <t>This property contains an alternative name for the Dataset. This property can be repeated for parallel language versions of the alternative name.</t>
-  </si>
-  <si>
-    <t>landing page</t>
-  </si>
-  <si>
-    <t>A web page that provides access to the Dataset, its Distributions and/or additional information.</t>
-  </si>
-  <si>
-    <t>It is intended to point to a landing page at the original data provider, not to a page on a site of a third party, such as an aggregator.</t>
-  </si>
-  <si>
-    <t>provenance</t>
-  </si>
-  <si>
-    <t>A statement about the lineage of a Dataset.</t>
-  </si>
-  <si>
-    <t>Information about how the data was collected, including methodologies, tools, and protocols used, this property can be repeated for different versions of the provenance (e.g. the provenance in different languages).</t>
-  </si>
-  <si>
-    <t>dct:provenance</t>
-  </si>
-  <si>
-    <t>dct:ProvenanceStatement</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="55" x14ac:knownFonts="1">
+  <fonts count="56" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3023,6 +3099,13 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="14">
     <fill>
@@ -3126,7 +3209,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="249">
+  <cellXfs count="250">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3812,25 +3895,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3839,20 +3937,8 @@
     <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3860,36 +3946,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="191">
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -3912,11 +3968,41 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4022,11 +4108,11 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="1"/>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4042,51 +4128,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color theme="1"/>
       </font>
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4145,8 +4191,58 @@
         <color rgb="FF9C5700"/>
       </font>
       <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4172,11 +4268,31 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4202,51 +4318,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color theme="1"/>
       </font>
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4292,11 +4368,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4312,11 +4388,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4332,6 +4408,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -4342,11 +4428,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
+        <color theme="1"/>
       </font>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
     </dxf>
@@ -7489,33 +7575,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>550</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>551</v>
+      </c>
+      <c r="N1" s="227" t="s">
+        <v>552</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>553</v>
-      </c>
-      <c r="M1" s="226" t="s">
-        <v>554</v>
-      </c>
-      <c r="N1" s="227" t="s">
-        <v>555</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>556</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="80" x14ac:dyDescent="0.2">
       <c r="A2" s="196" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="B2" s="45" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="C2" s="76" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="D2" s="196" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="197" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="F2" s="198" t="s">
         <v>35</v>
@@ -7524,7 +7610,7 @@
         <v>58</v>
       </c>
       <c r="H2" s="198" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="I2" s="160" t="s">
         <v>20</v>
@@ -7539,13 +7625,13 @@
     </row>
     <row r="3" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="68" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="D3" s="68" t="s">
         <v>16</v>
@@ -7684,36 +7770,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>562</v>
+      </c>
+      <c r="M1" s="220" t="s">
+        <v>563</v>
+      </c>
+      <c r="N1" s="226" t="s">
+        <v>564</v>
+      </c>
+      <c r="O1" s="230" t="s">
         <v>565</v>
       </c>
-      <c r="M1" s="220" t="s">
+      <c r="P1" s="227" t="s">
         <v>566</v>
       </c>
-      <c r="N1" s="226" t="s">
+      <c r="Q1" s="231" t="s">
         <v>567</v>
       </c>
-      <c r="O1" s="230" t="s">
+      <c r="R1" s="233" t="s">
         <v>568</v>
-      </c>
-      <c r="P1" s="227" t="s">
-        <v>569</v>
-      </c>
-      <c r="Q1" s="231" t="s">
-        <v>570</v>
-      </c>
-      <c r="R1" s="233" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="58" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="C2" s="76" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
@@ -7741,13 +7827,13 @@
     </row>
     <row r="3" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8409,33 +8495,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>575</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>576</v>
+      </c>
+      <c r="N1" s="227" t="s">
+        <v>577</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>578</v>
-      </c>
-      <c r="M1" s="226" t="s">
-        <v>579</v>
-      </c>
-      <c r="N1" s="227" t="s">
-        <v>580</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="84" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8465,19 +8551,19 @@
     </row>
     <row r="3" spans="1:15" ht="144" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
+        <v>583</v>
+      </c>
+      <c r="B3" s="49" t="s">
+        <v>584</v>
+      </c>
+      <c r="C3" s="77" t="s">
+        <v>585</v>
+      </c>
+      <c r="D3" s="234" t="s">
         <v>586</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="E3" s="50" t="s">
         <v>587</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>588</v>
-      </c>
-      <c r="D3" s="234" t="s">
-        <v>589</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>590</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8603,33 +8689,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="218" t="s">
+        <v>588</v>
+      </c>
+      <c r="M1" s="229" t="s">
+        <v>589</v>
+      </c>
+      <c r="N1" s="228" t="s">
+        <v>590</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>591</v>
-      </c>
-      <c r="M1" s="229" t="s">
-        <v>592</v>
-      </c>
-      <c r="N1" s="228" t="s">
-        <v>593</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>594</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="160" x14ac:dyDescent="0.2">
       <c r="A2" s="84" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="D2" s="59" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>35</v>
@@ -8650,19 +8736,19 @@
     </row>
     <row r="3" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>35</v>
@@ -8788,33 +8874,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>599</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>600</v>
+      </c>
+      <c r="N1" s="227" t="s">
+        <v>601</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>602</v>
-      </c>
-      <c r="M1" s="226" t="s">
-        <v>603</v>
-      </c>
-      <c r="N1" s="227" t="s">
-        <v>604</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>605</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="112" x14ac:dyDescent="0.2">
       <c r="A2" s="84" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8835,19 +8921,19 @@
     </row>
     <row r="3" spans="1:15" ht="64" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8951,7 +9037,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="E1" s="56" t="s">
         <v>4</v>
@@ -8974,13 +9060,13 @@
     </row>
     <row r="2" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="63" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="D2" s="43" t="s">
         <v>16</v>
@@ -8988,7 +9074,7 @@
       <c r="E2" s="45"/>
       <c r="F2" s="64"/>
       <c r="G2" s="63" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="H2" s="65" t="s">
         <v>81</v>
@@ -9002,13 +9088,13 @@
     </row>
     <row r="3" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="67" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="B3" s="50" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C3" s="49" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -9016,10 +9102,10 @@
       <c r="E3" s="50"/>
       <c r="F3" s="68"/>
       <c r="G3" s="69" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="H3" s="48" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="I3" s="69" t="s">
         <v>20</v>
@@ -9030,13 +9116,13 @@
     </row>
     <row r="4" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="63" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>16</v>
@@ -9044,10 +9130,10 @@
       <c r="E4" s="53"/>
       <c r="F4" s="64"/>
       <c r="G4" s="63" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="H4" s="65" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="I4" s="66" t="s">
         <v>20</v>
@@ -9058,26 +9144,26 @@
     </row>
     <row r="5" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="67" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="B5" s="50" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="C5" s="49" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="D5" s="48" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="F5" s="68"/>
       <c r="G5" s="67" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="H5" s="48" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="I5" s="69" t="s">
         <v>20</v>
@@ -9088,13 +9174,13 @@
     </row>
     <row r="6" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="63" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="B6" s="73" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>16</v>
@@ -9105,7 +9191,7 @@
         <v>98</v>
       </c>
       <c r="H6" s="65" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="I6" s="66" t="s">
         <v>20</v>
@@ -9116,13 +9202,13 @@
     </row>
     <row r="7" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="67" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="C7" s="49" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>16</v>
@@ -9144,23 +9230,23 @@
     </row>
     <row r="8" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A8" s="63" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="71" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="F8" s="47"/>
       <c r="G8" s="63" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="H8" s="65">
         <v>1</v>
@@ -9174,13 +9260,13 @@
     </row>
     <row r="9" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="67" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C9" s="49" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="D9" s="48" t="s">
         <v>16</v>
@@ -9188,7 +9274,7 @@
       <c r="E9" s="50"/>
       <c r="F9" s="68"/>
       <c r="G9" s="69" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="H9" s="48" t="s">
         <v>81</v>
@@ -9202,23 +9288,23 @@
     </row>
     <row r="10" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="63" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="B10" s="72" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="72" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="F10" s="64"/>
       <c r="G10" s="63" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="H10" s="65" t="s">
         <v>19</v>
@@ -9514,42 +9600,42 @@
     <cfRule type="cellIs" dxfId="49" priority="41" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="42" operator="equal">
-      <formula>"Recommended"</formula>
+    <cfRule type="cellIs" dxfId="48" priority="44" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="47" priority="43" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="44" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="46" priority="42" operator="equal">
+      <formula>"Recommended"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D26:E28">
-    <cfRule type="cellIs" dxfId="45" priority="45" operator="equal">
-      <formula>"Optional"</formula>
+    <cfRule type="cellIs" dxfId="45" priority="48" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="47" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="46" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="47" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="48" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="42" priority="45" operator="equal">
+      <formula>"Optional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="cellIs" dxfId="41" priority="51" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="54" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="51" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="52" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="52" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="53" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="53" operator="equal">
       <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="54" operator="equal">
-      <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F7 E8">
@@ -9558,28 +9644,28 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9:F38">
-    <cfRule type="cellIs" dxfId="36" priority="33" operator="equal">
-      <formula>"Not added"</formula>
+    <cfRule type="cellIs" dxfId="36" priority="38" operator="equal">
+      <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="36" operator="equal">
-      <formula>"Optional"</formula>
+    <cfRule type="cellIs" dxfId="35" priority="39" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="34" priority="37" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="38" operator="equal">
-      <formula>"Mandatory"</formula>
+    <cfRule type="cellIs" dxfId="33" priority="36" operator="equal">
+      <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="39" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="32" priority="33" operator="equal">
+      <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H11">
-    <cfRule type="cellIs" dxfId="31" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="31" priority="10" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="9" operator="greaterThan">
       <formula>"reviewd"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="10" operator="equal">
-      <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14:H27 H36:H38">
@@ -9591,17 +9677,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F7">
-    <cfRule type="cellIs" dxfId="27" priority="15" operator="equal">
-      <formula>"Optional"</formula>
+    <cfRule type="cellIs" dxfId="27" priority="18" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="17" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="16" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="17" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="18" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="24" priority="15" operator="equal">
+      <formula>"Optional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -9683,36 +9769,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="M1" s="226" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="N1" s="233" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A2" s="44" t="s">
+        <v>654</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>655</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>656</v>
+      </c>
+      <c r="D2" s="78" t="s">
         <v>657</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="E2" s="197" t="s">
         <v>658</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>659</v>
-      </c>
-      <c r="D2" s="78" t="s">
-        <v>660</v>
-      </c>
-      <c r="E2" s="197" t="s">
-        <v>661</v>
       </c>
       <c r="F2" s="46" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="204" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="H2" s="47">
         <v>1</v>
@@ -9726,13 +9812,13 @@
     </row>
     <row r="3" spans="1:14" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="49" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="C3" s="48" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="D3" s="50" t="s">
         <v>16</v>
@@ -9742,7 +9828,7 @@
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="H3" s="52">
         <v>1</v>
@@ -10261,14 +10347,14 @@
     <cfRule type="cellIs" dxfId="19" priority="25" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="26" operator="equal">
-      <formula>"Recommended"</formula>
+    <cfRule type="cellIs" dxfId="18" priority="28" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="17" priority="27" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="28" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="16" priority="26" operator="equal">
+      <formula>"Recommended"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E3">
@@ -10308,25 +10394,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="5" priority="29" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="30" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="29" operator="greaterThan">
       <formula>"reviewd"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="30" operator="equal">
-      <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F52">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
-      <formula>"Optional"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"Optional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -10656,13 +10742,13 @@
       <c r="M7" s="129"/>
     </row>
     <row r="8" spans="1:13" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="237" t="s">
+      <c r="A8" s="236" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="238" t="s">
+      <c r="B8" s="242" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="237" t="s">
+      <c r="C8" s="236" t="s">
         <v>62</v>
       </c>
       <c r="D8" s="213" t="s">
@@ -10671,92 +10757,92 @@
       <c r="E8" s="239" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="236" t="s">
+      <c r="F8" s="238" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="236" t="s">
+      <c r="G8" s="238" t="s">
         <v>65</v>
       </c>
-      <c r="H8" s="236" t="s">
+      <c r="H8" s="238" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="235" t="s">
+      <c r="I8" s="240" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="235" t="s">
+      <c r="J8" s="240" t="s">
         <v>66</v>
       </c>
       <c r="K8" s="137"/>
-      <c r="L8" s="235"/>
-      <c r="M8" s="235"/>
+      <c r="L8" s="240"/>
+      <c r="M8" s="240"/>
     </row>
     <row r="9" spans="1:13" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="237"/>
-      <c r="B9" s="238"/>
-      <c r="C9" s="237"/>
+      <c r="A9" s="236"/>
+      <c r="B9" s="242"/>
+      <c r="C9" s="236"/>
       <c r="D9" s="214" t="s">
         <v>67</v>
       </c>
       <c r="E9" s="239"/>
-      <c r="F9" s="236"/>
-      <c r="G9" s="236"/>
-      <c r="H9" s="236"/>
-      <c r="I9" s="235"/>
-      <c r="J9" s="235"/>
+      <c r="F9" s="238"/>
+      <c r="G9" s="238"/>
+      <c r="H9" s="238"/>
+      <c r="I9" s="240"/>
+      <c r="J9" s="240"/>
       <c r="K9" s="137"/>
-      <c r="L9" s="235"/>
-      <c r="M9" s="235"/>
+      <c r="L9" s="240"/>
+      <c r="M9" s="240"/>
     </row>
     <row r="10" spans="1:13" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="237"/>
-      <c r="B10" s="238"/>
-      <c r="C10" s="237"/>
+      <c r="A10" s="236"/>
+      <c r="B10" s="242"/>
+      <c r="C10" s="236"/>
       <c r="D10" s="214" t="s">
         <v>68</v>
       </c>
       <c r="E10" s="239"/>
-      <c r="F10" s="236"/>
-      <c r="G10" s="236"/>
-      <c r="H10" s="236"/>
-      <c r="I10" s="235"/>
-      <c r="J10" s="235"/>
+      <c r="F10" s="238"/>
+      <c r="G10" s="238"/>
+      <c r="H10" s="238"/>
+      <c r="I10" s="240"/>
+      <c r="J10" s="240"/>
       <c r="K10" s="137"/>
-      <c r="L10" s="235"/>
-      <c r="M10" s="235"/>
+      <c r="L10" s="240"/>
+      <c r="M10" s="240"/>
     </row>
     <row r="11" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="237"/>
-      <c r="B11" s="238"/>
-      <c r="C11" s="237"/>
+      <c r="A11" s="236"/>
+      <c r="B11" s="242"/>
+      <c r="C11" s="236"/>
       <c r="D11" s="152" t="s">
         <v>69</v>
       </c>
       <c r="E11" s="239"/>
-      <c r="F11" s="236"/>
-      <c r="G11" s="236"/>
-      <c r="H11" s="236"/>
-      <c r="I11" s="235"/>
-      <c r="J11" s="235"/>
+      <c r="F11" s="238"/>
+      <c r="G11" s="238"/>
+      <c r="H11" s="238"/>
+      <c r="I11" s="240"/>
+      <c r="J11" s="240"/>
       <c r="K11" s="153"/>
-      <c r="L11" s="235"/>
-      <c r="M11" s="235"/>
+      <c r="L11" s="240"/>
+      <c r="M11" s="240"/>
     </row>
     <row r="12" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="237"/>
-      <c r="B12" s="238"/>
-      <c r="C12" s="237"/>
+      <c r="A12" s="236"/>
+      <c r="B12" s="242"/>
+      <c r="C12" s="236"/>
       <c r="D12" s="152" t="s">
         <v>70</v>
       </c>
       <c r="E12" s="239"/>
-      <c r="F12" s="236"/>
-      <c r="G12" s="236"/>
-      <c r="H12" s="236"/>
-      <c r="I12" s="235"/>
-      <c r="J12" s="235"/>
+      <c r="F12" s="238"/>
+      <c r="G12" s="238"/>
+      <c r="H12" s="238"/>
+      <c r="I12" s="240"/>
+      <c r="J12" s="240"/>
       <c r="K12" s="137"/>
-      <c r="L12" s="235"/>
-      <c r="M12" s="235"/>
+      <c r="L12" s="240"/>
+      <c r="M12" s="240"/>
     </row>
     <row r="13" spans="1:13" ht="48" x14ac:dyDescent="0.2">
       <c r="A13" s="125" t="s">
@@ -10881,7 +10967,7 @@
         <v>92</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -11575,17 +11661,17 @@
     <sortCondition ref="A2:A24"/>
   </sortState>
   <mergeCells count="11">
+    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="L8:L12"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I8:I12"/>
+    <mergeCell ref="J8:J12"/>
     <mergeCell ref="G8:G12"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="F8:F12"/>
-    <mergeCell ref="M8:M12"/>
-    <mergeCell ref="L8:L12"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="J8:J12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="cellIs" dxfId="190" priority="16" operator="equal">
@@ -11805,19 +11891,19 @@
     </row>
     <row r="3" spans="1:14" ht="209.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="121" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="C3" s="121" t="s">
-        <v>678</v>
-      </c>
-      <c r="D3" s="248" t="s">
+        <v>674</v>
+      </c>
+      <c r="D3" s="235" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="123" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="F3" s="124" t="s">
         <v>17</v>
@@ -11891,7 +11977,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="132" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="F5" s="124" t="s">
         <v>35</v>
@@ -12266,13 +12352,13 @@
       <c r="N14" s="129"/>
     </row>
     <row r="15" spans="1:14" ht="32" x14ac:dyDescent="0.2">
-      <c r="A15" s="237" t="s">
+      <c r="A15" s="236" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="241" t="s">
+      <c r="B15" s="237" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="237" t="s">
+      <c r="C15" s="236" t="s">
         <v>62</v>
       </c>
       <c r="D15" s="213" t="s">
@@ -12281,87 +12367,87 @@
       <c r="E15" s="239" t="s">
         <v>199</v>
       </c>
-      <c r="F15" s="236" t="s">
+      <c r="F15" s="238" t="s">
         <v>17</v>
       </c>
-      <c r="G15" s="236" t="s">
+      <c r="G15" s="238" t="s">
         <v>65</v>
       </c>
-      <c r="H15" s="236" t="s">
+      <c r="H15" s="238" t="s">
         <v>19</v>
       </c>
-      <c r="I15" s="235" t="s">
+      <c r="I15" s="240" t="s">
         <v>20</v>
       </c>
-      <c r="J15" s="235" t="s">
+      <c r="J15" s="240" t="s">
         <v>66</v>
       </c>
-      <c r="K15" s="240"/>
-      <c r="L15" s="235"/>
+      <c r="K15" s="241"/>
+      <c r="L15" s="240"/>
     </row>
     <row r="16" spans="1:14" ht="32" x14ac:dyDescent="0.2">
-      <c r="A16" s="237"/>
-      <c r="B16" s="241"/>
-      <c r="C16" s="237"/>
+      <c r="A16" s="236"/>
+      <c r="B16" s="237"/>
+      <c r="C16" s="236"/>
       <c r="D16" s="214" t="s">
         <v>67</v>
       </c>
       <c r="E16" s="239"/>
-      <c r="F16" s="236"/>
-      <c r="G16" s="236"/>
-      <c r="H16" s="236"/>
-      <c r="I16" s="235"/>
-      <c r="J16" s="235"/>
-      <c r="K16" s="240"/>
-      <c r="L16" s="235"/>
+      <c r="F16" s="238"/>
+      <c r="G16" s="238"/>
+      <c r="H16" s="238"/>
+      <c r="I16" s="240"/>
+      <c r="J16" s="240"/>
+      <c r="K16" s="241"/>
+      <c r="L16" s="240"/>
     </row>
     <row r="17" spans="1:14" ht="32" x14ac:dyDescent="0.2">
-      <c r="A17" s="237"/>
-      <c r="B17" s="241"/>
-      <c r="C17" s="237"/>
+      <c r="A17" s="236"/>
+      <c r="B17" s="237"/>
+      <c r="C17" s="236"/>
       <c r="D17" s="214" t="s">
         <v>68</v>
       </c>
       <c r="E17" s="239"/>
-      <c r="F17" s="236"/>
-      <c r="G17" s="236"/>
-      <c r="H17" s="236"/>
-      <c r="I17" s="235"/>
-      <c r="J17" s="235"/>
-      <c r="K17" s="240"/>
-      <c r="L17" s="235"/>
+      <c r="F17" s="238"/>
+      <c r="G17" s="238"/>
+      <c r="H17" s="238"/>
+      <c r="I17" s="240"/>
+      <c r="J17" s="240"/>
+      <c r="K17" s="241"/>
+      <c r="L17" s="240"/>
     </row>
     <row r="18" spans="1:14" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="237"/>
-      <c r="B18" s="241"/>
-      <c r="C18" s="237"/>
+      <c r="A18" s="236"/>
+      <c r="B18" s="237"/>
+      <c r="C18" s="236"/>
       <c r="D18" s="152" t="s">
         <v>69</v>
       </c>
       <c r="E18" s="239"/>
-      <c r="F18" s="236"/>
-      <c r="G18" s="236"/>
-      <c r="H18" s="236"/>
-      <c r="I18" s="235"/>
-      <c r="J18" s="235"/>
-      <c r="K18" s="240"/>
-      <c r="L18" s="235"/>
+      <c r="F18" s="238"/>
+      <c r="G18" s="238"/>
+      <c r="H18" s="238"/>
+      <c r="I18" s="240"/>
+      <c r="J18" s="240"/>
+      <c r="K18" s="241"/>
+      <c r="L18" s="240"/>
     </row>
     <row r="19" spans="1:14" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="237"/>
-      <c r="B19" s="241"/>
-      <c r="C19" s="237"/>
+      <c r="A19" s="236"/>
+      <c r="B19" s="237"/>
+      <c r="C19" s="236"/>
       <c r="D19" s="152" t="s">
         <v>70</v>
       </c>
       <c r="E19" s="239"/>
-      <c r="F19" s="236"/>
-      <c r="G19" s="236"/>
-      <c r="H19" s="236"/>
-      <c r="I19" s="235"/>
-      <c r="J19" s="235"/>
-      <c r="K19" s="240"/>
-      <c r="L19" s="235"/>
+      <c r="F19" s="238"/>
+      <c r="G19" s="238"/>
+      <c r="H19" s="238"/>
+      <c r="I19" s="240"/>
+      <c r="J19" s="240"/>
+      <c r="K19" s="241"/>
+      <c r="L19" s="240"/>
     </row>
     <row r="20" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="125" t="s">
@@ -12589,19 +12675,19 @@
     </row>
     <row r="26" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="121" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="B26" s="35" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="C26" s="141" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="D26" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E26" s="71" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="F26" s="124" t="s">
         <v>17</v>
@@ -12673,7 +12759,7 @@
         <v>237</v>
       </c>
       <c r="E28" s="132" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="F28" s="124" t="s">
         <v>17</v>
@@ -12993,25 +13079,25 @@
     </row>
     <row r="37" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="121" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="B37" s="35" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="C37" s="121" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="D37" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E37" s="132" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="F37" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G37" s="124" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
       <c r="H37" s="124" t="s">
         <v>19</v>
@@ -13083,7 +13169,7 @@
         <v>285</v>
       </c>
       <c r="E39" s="138" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="F39" s="124" t="s">
         <v>17</v>
@@ -13283,7 +13369,7 @@
         <v>16</v>
       </c>
       <c r="E44" s="74" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="F44" s="127" t="s">
         <v>17</v>
@@ -13757,17 +13843,17 @@
     <sortCondition ref="A2:A56"/>
   </sortState>
   <mergeCells count="11">
-    <mergeCell ref="A15:A19"/>
-    <mergeCell ref="B15:B19"/>
-    <mergeCell ref="C15:C19"/>
-    <mergeCell ref="F15:F19"/>
-    <mergeCell ref="E15:E19"/>
     <mergeCell ref="L15:L19"/>
     <mergeCell ref="K15:K19"/>
     <mergeCell ref="G15:G19"/>
     <mergeCell ref="H15:H19"/>
     <mergeCell ref="I15:I19"/>
     <mergeCell ref="J15:J19"/>
+    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="B15:B19"/>
+    <mergeCell ref="C15:C19"/>
+    <mergeCell ref="F15:F19"/>
+    <mergeCell ref="E15:E19"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F15 F20:F56">
     <cfRule type="cellIs" dxfId="171" priority="8" operator="equal">
@@ -13967,7 +14053,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="64" t="s">
         <v>364</v>
       </c>
@@ -13980,8 +14066,8 @@
       <c r="D2" s="152" t="s">
         <v>365</v>
       </c>
-      <c r="E2" s="158" t="s">
-        <v>366</v>
+      <c r="E2" s="249" t="s">
+        <v>684</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
@@ -14001,25 +14087,25 @@
     </row>
     <row r="3" spans="1:22" ht="128" x14ac:dyDescent="0.2">
       <c r="A3" s="68" t="s">
+        <v>366</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>367</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="68" t="s">
         <v>368</v>
-      </c>
-      <c r="C3" s="68" t="s">
-        <v>369</v>
       </c>
       <c r="D3" s="162" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -14031,7 +14117,7 @@
         <v>66</v>
       </c>
       <c r="K3" s="136" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -14055,10 +14141,10 @@
         <v>213</v>
       </c>
       <c r="D4" s="71" t="s">
+        <v>371</v>
+      </c>
+      <c r="E4" s="158" t="s">
         <v>372</v>
-      </c>
-      <c r="E4" s="158" t="s">
-        <v>373</v>
       </c>
       <c r="F4" s="159" t="s">
         <v>35</v>
@@ -14073,28 +14159,28 @@
         <v>28</v>
       </c>
       <c r="J4" s="160" t="s">
+        <v>373</v>
+      </c>
+      <c r="K4" s="136" t="s">
         <v>374</v>
-      </c>
-      <c r="K4" s="136" t="s">
-        <v>375</v>
       </c>
       <c r="L4" s="107"/>
     </row>
     <row r="5" spans="1:22" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="165" t="s">
+        <v>375</v>
+      </c>
+      <c r="B5" s="75" t="s">
         <v>376</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="C5" s="165" t="s">
         <v>377</v>
-      </c>
-      <c r="C5" s="165" t="s">
-        <v>378</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="75" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F5" s="166" t="s">
         <v>35</v>
@@ -14112,7 +14198,7 @@
         <v>29</v>
       </c>
       <c r="K5" s="136" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
@@ -14125,21 +14211,21 @@
       <c r="T5" s="129"/>
       <c r="U5" s="129"/>
     </row>
-    <row r="6" spans="1:22" ht="80" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" ht="96" x14ac:dyDescent="0.2">
       <c r="A6" s="168" t="s">
+        <v>380</v>
+      </c>
+      <c r="B6" s="151" t="s">
         <v>381</v>
       </c>
-      <c r="B6" s="151" t="s">
+      <c r="C6" s="168" t="s">
         <v>382</v>
-      </c>
-      <c r="C6" s="168" t="s">
-        <v>383</v>
       </c>
       <c r="D6" s="169" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="151" t="s">
-        <v>384</v>
+        <v>685</v>
       </c>
       <c r="F6" s="133" t="s">
         <v>17</v>
@@ -14159,21 +14245,21 @@
       <c r="K6" s="161"/>
       <c r="L6" s="107"/>
     </row>
-    <row r="7" spans="1:22" ht="128" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" ht="144" x14ac:dyDescent="0.2">
       <c r="A7" s="125" t="s">
+        <v>383</v>
+      </c>
+      <c r="B7" s="74" t="s">
+        <v>384</v>
+      </c>
+      <c r="C7" s="125" t="s">
         <v>385</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="D7" s="171" t="s">
         <v>386</v>
       </c>
-      <c r="C7" s="125" t="s">
-        <v>387</v>
-      </c>
-      <c r="D7" s="171" t="s">
-        <v>388</v>
-      </c>
       <c r="E7" s="81" t="s">
-        <v>389</v>
+        <v>686</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
@@ -14213,10 +14299,10 @@
         <v>338</v>
       </c>
       <c r="D8" s="143" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="E8" s="135" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="F8" s="159" t="s">
         <v>17</v>
@@ -14234,13 +14320,13 @@
         <v>29</v>
       </c>
       <c r="K8" s="136" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:22" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="165" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="B9" s="75" t="s">
         <v>77</v>
@@ -14252,7 +14338,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="173" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="F9" s="166" t="s">
         <v>35</v>
@@ -14270,7 +14356,7 @@
         <v>66</v>
       </c>
       <c r="K9" s="136" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
@@ -15015,45 +15101,45 @@
         <v>10</v>
       </c>
       <c r="L1" s="225" t="s">
+        <v>392</v>
+      </c>
+      <c r="M1" s="108" t="s">
+        <v>393</v>
+      </c>
+      <c r="N1" s="223" t="s">
+        <v>394</v>
+      </c>
+      <c r="O1" s="224" t="s">
         <v>395</v>
       </c>
-      <c r="M1" s="108" t="s">
+      <c r="P1" s="232" t="s">
         <v>396</v>
       </c>
-      <c r="N1" s="223" t="s">
+      <c r="Q1" s="233" t="s">
         <v>397</v>
-      </c>
-      <c r="O1" s="224" t="s">
-        <v>398</v>
-      </c>
-      <c r="P1" s="232" t="s">
-        <v>399</v>
-      </c>
-      <c r="Q1" s="233" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="64.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="64" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="B2" s="45" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="C2" s="172" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="D2" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="88" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="159" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="H2" s="159" t="s">
         <v>19</v>
@@ -15065,31 +15151,31 @@
         <v>29</v>
       </c>
       <c r="K2" s="156" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="L2" s="136"/>
     </row>
     <row r="3" spans="1:17" ht="128" x14ac:dyDescent="0.2">
       <c r="A3" s="68" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C3" s="68" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="D3" s="183" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -15101,7 +15187,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="156" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="L3" s="75"/>
       <c r="M3" s="61"/>
@@ -15111,28 +15197,28 @@
     </row>
     <row r="4" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="64" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C4" s="64" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="D4" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="88" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="F4" s="159" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="G4" s="159" t="s">
-        <v>414</v>
-      </c>
-      <c r="H4" s="159">
-        <v>1</v>
+        <v>411</v>
+      </c>
+      <c r="H4" s="159" t="s">
+        <v>81</v>
       </c>
       <c r="I4" s="160" t="s">
         <v>28</v>
@@ -15141,7 +15227,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="156" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="L4" s="136"/>
     </row>
@@ -15964,27 +16050,27 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="M1" s="223" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="121" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B2" s="35" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C2" s="121" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="D2" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -16002,30 +16088,30 @@
         <v>37</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="L2" s="141" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="M2" s="141" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="64" x14ac:dyDescent="0.2">
       <c r="A3" s="125" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="B3" s="74" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="C3" s="125" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="D3" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="85" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="F3" s="127" t="s">
         <v>35</v>
@@ -16043,7 +16129,7 @@
         <v>37</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -16062,7 +16148,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="35" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -16087,28 +16173,28 @@
     </row>
     <row r="5" spans="1:13" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="125" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="B5" s="74" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="C5" s="134" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="126" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="F5" s="127" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="G5" s="127" t="s">
-        <v>434</v>
-      </c>
-      <c r="H5" s="127">
-        <v>1</v>
+        <v>431</v>
+      </c>
+      <c r="H5" s="127" t="s">
+        <v>81</v>
       </c>
       <c r="I5" s="129" t="s">
         <v>20</v>
@@ -16117,32 +16203,32 @@
         <v>29</v>
       </c>
       <c r="K5" s="98" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
     </row>
     <row r="6" spans="1:13" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" s="121" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="C6" s="121" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="D6" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="F6" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="128" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="H6" s="124" t="s">
         <v>81</v>
@@ -16154,36 +16240,36 @@
         <v>29</v>
       </c>
       <c r="K6" s="98" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="L6" s="107" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="M6" s="107" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" s="125" t="s">
+        <v>440</v>
+      </c>
+      <c r="B7" s="74" t="s">
+        <v>441</v>
+      </c>
+      <c r="C7" s="134" t="s">
+        <v>442</v>
+      </c>
+      <c r="D7" s="185" t="s">
         <v>443</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="E7" s="126" t="s">
         <v>444</v>
-      </c>
-      <c r="C7" s="134" t="s">
-        <v>445</v>
-      </c>
-      <c r="D7" s="185" t="s">
-        <v>446</v>
-      </c>
-      <c r="E7" s="126" t="s">
-        <v>447</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="156" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="H7" s="127" t="s">
         <v>81</v>
@@ -16195,7 +16281,7 @@
         <v>29</v>
       </c>
       <c r="K7" s="98" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="L7" s="129"/>
       <c r="M7" s="129"/>
@@ -16214,7 +16300,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>17</v>
@@ -16232,7 +16318,7 @@
         <v>29</v>
       </c>
       <c r="K8" s="98" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="L8" s="107"/>
       <c r="M8" s="107"/>
@@ -16251,7 +16337,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="126" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>17</v>
@@ -16269,26 +16355,26 @@
         <v>29</v>
       </c>
       <c r="K9" s="98" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
     </row>
     <row r="10" spans="1:13" ht="48" x14ac:dyDescent="0.2">
       <c r="A10" s="121" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="C10" s="141" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>17</v>
@@ -16306,35 +16392,35 @@
         <v>37</v>
       </c>
       <c r="K10" s="98" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="L10" s="107"/>
       <c r="M10" s="107"/>
     </row>
     <row r="11" spans="1:13" ht="48" x14ac:dyDescent="0.2">
       <c r="A11" s="125" t="s">
+        <v>456</v>
+      </c>
+      <c r="B11" s="74" t="s">
+        <v>457</v>
+      </c>
+      <c r="C11" s="125" t="s">
+        <v>458</v>
+      </c>
+      <c r="D11" s="154" t="s">
         <v>459</v>
       </c>
-      <c r="B11" s="74" t="s">
+      <c r="E11" s="126" t="s">
+        <v>667</v>
+      </c>
+      <c r="F11" s="127" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="127" t="s">
         <v>460</v>
       </c>
-      <c r="C11" s="125" t="s">
-        <v>461</v>
-      </c>
-      <c r="D11" s="154" t="s">
-        <v>462</v>
-      </c>
-      <c r="E11" s="126" t="s">
-        <v>670</v>
-      </c>
-      <c r="F11" s="127" t="s">
-        <v>35</v>
-      </c>
-      <c r="G11" s="127" t="s">
-        <v>463</v>
-      </c>
-      <c r="H11" s="127">
-        <v>1</v>
+      <c r="H11" s="127" t="s">
+        <v>81</v>
       </c>
       <c r="I11" s="129" t="s">
         <v>20</v>
@@ -16343,7 +16429,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="L11" s="129"/>
       <c r="M11" s="129"/>
@@ -16362,7 +16448,7 @@
         <v>85</v>
       </c>
       <c r="E12" s="138" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -16380,14 +16466,14 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="L12" s="107"/>
       <c r="M12" s="107"/>
     </row>
     <row r="13" spans="1:13" ht="80" x14ac:dyDescent="0.2">
       <c r="A13" s="125" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="B13" s="74" t="s">
         <v>90</v>
@@ -16399,13 +16485,13 @@
         <v>92</v>
       </c>
       <c r="E13" s="80" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G13" s="127" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="H13" s="127">
         <v>1</v>
@@ -16417,14 +16503,14 @@
         <v>37</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="L13" s="129"/>
       <c r="M13" s="129"/>
     </row>
     <row r="14" spans="1:13" ht="80" x14ac:dyDescent="0.2">
       <c r="A14" s="121" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="B14" s="35" t="s">
         <v>175</v>
@@ -16436,7 +16522,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -16454,32 +16540,32 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="L14" s="107"/>
       <c r="M14" s="107"/>
     </row>
     <row r="15" spans="1:13" ht="112" x14ac:dyDescent="0.2">
       <c r="A15" s="125" t="s">
+        <v>471</v>
+      </c>
+      <c r="B15" s="74" t="s">
+        <v>472</v>
+      </c>
+      <c r="C15" s="125" t="s">
+        <v>473</v>
+      </c>
+      <c r="D15" s="185" t="s">
+        <v>443</v>
+      </c>
+      <c r="E15" s="80" t="s">
         <v>474</v>
-      </c>
-      <c r="B15" s="74" t="s">
-        <v>475</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>476</v>
-      </c>
-      <c r="D15" s="185" t="s">
-        <v>446</v>
-      </c>
-      <c r="E15" s="80" t="s">
-        <v>477</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G15" s="127" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="H15" s="127" t="s">
         <v>81</v>
@@ -16491,7 +16577,7 @@
         <v>29</v>
       </c>
       <c r="K15" s="98" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="L15" s="129"/>
       <c r="M15" s="129"/>
@@ -16526,32 +16612,32 @@
         <v>29</v>
       </c>
       <c r="K16" s="98" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="L16" s="107"/>
       <c r="M16" s="107"/>
     </row>
     <row r="17" spans="1:13" ht="48" x14ac:dyDescent="0.2">
       <c r="A17" s="125" t="s">
+        <v>477</v>
+      </c>
+      <c r="B17" s="74" t="s">
+        <v>478</v>
+      </c>
+      <c r="C17" s="125" t="s">
+        <v>479</v>
+      </c>
+      <c r="D17" s="185" t="s">
+        <v>443</v>
+      </c>
+      <c r="E17" s="74" t="s">
         <v>480</v>
-      </c>
-      <c r="B17" s="74" t="s">
-        <v>481</v>
-      </c>
-      <c r="C17" s="125" t="s">
-        <v>482</v>
-      </c>
-      <c r="D17" s="185" t="s">
-        <v>446</v>
-      </c>
-      <c r="E17" s="74" t="s">
-        <v>483</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G17" s="127" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="H17" s="127" t="s">
         <v>81</v>
@@ -16563,7 +16649,7 @@
         <v>29</v>
       </c>
       <c r="K17" s="98" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="L17" s="129"/>
       <c r="M17" s="129"/>
@@ -16582,7 +16668,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="132" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -16600,12 +16686,12 @@
         <v>29</v>
       </c>
       <c r="K18" s="98" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="L18" s="107"/>
       <c r="M18" s="107"/>
     </row>
-    <row r="19" spans="1:13" ht="185.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="231" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="125" t="s">
         <v>306</v>
       </c>
@@ -16613,11 +16699,11 @@
         <v>307</v>
       </c>
       <c r="C19" s="125" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="D19" s="126"/>
       <c r="E19" s="74" t="s">
-        <v>675</v>
+        <v>687</v>
       </c>
       <c r="F19" s="127" t="s">
         <v>17</v>
@@ -16636,10 +16722,10 @@
       </c>
       <c r="K19" s="104"/>
       <c r="L19" s="129" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="M19" s="129" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="144" x14ac:dyDescent="0.2">
@@ -16656,16 +16742,16 @@
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="F20" s="190" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="G20" s="124" t="s">
         <v>114</v>
       </c>
-      <c r="H20" s="133">
-        <v>1</v>
+      <c r="H20" s="133" t="s">
+        <v>81</v>
       </c>
       <c r="I20" s="107" t="s">
         <v>20</v>
@@ -16674,7 +16760,7 @@
         <v>29</v>
       </c>
       <c r="K20" s="99" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="L20" s="107"/>
       <c r="M20" s="107"/>
@@ -16690,10 +16776,10 @@
         <v>322</v>
       </c>
       <c r="D21" s="154" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="E21" s="81" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -16711,7 +16797,7 @@
         <v>29</v>
       </c>
       <c r="K21" s="98" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
@@ -16730,7 +16816,7 @@
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
@@ -16765,7 +16851,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
@@ -16783,7 +16869,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="98" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -17265,7 +17351,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -17282,7 +17368,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="74" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -17300,7 +17386,7 @@
         <v>29</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="L2" s="129"/>
     </row>
@@ -17321,13 +17407,13 @@
         <v>34</v>
       </c>
       <c r="F3" s="124" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="G3" s="128" t="s">
         <v>36</v>
       </c>
       <c r="H3" s="124" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="I3" s="107" t="s">
         <v>104</v>
@@ -17336,7 +17422,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="L3" s="107" t="s">
         <v>39</v>
@@ -17356,7 +17442,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="126" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="F4" s="127" t="s">
         <v>35</v>
@@ -17374,7 +17460,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="99" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="L4" s="129"/>
     </row>
@@ -17392,7 +17478,7 @@
         <v>196</v>
       </c>
       <c r="E5" s="135" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="F5" s="124" t="s">
         <v>17</v>
@@ -17413,104 +17499,104 @@
       <c r="L5" s="107"/>
     </row>
     <row r="6" spans="1:12" ht="32" x14ac:dyDescent="0.2">
-      <c r="A6" s="245" t="s">
+      <c r="A6" s="244" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="246" t="s">
+      <c r="B6" s="245" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="245" t="s">
+      <c r="C6" s="244" t="s">
         <v>62</v>
       </c>
       <c r="D6" s="215" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="247" t="s">
+      <c r="E6" s="246" t="s">
         <v>199</v>
       </c>
-      <c r="F6" s="244" t="s">
+      <c r="F6" s="243" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="244" t="s">
+      <c r="G6" s="243" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="244" t="s">
+      <c r="H6" s="243" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="242" t="s">
+      <c r="I6" s="247" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="235" t="s">
+      <c r="J6" s="240" t="s">
         <v>66</v>
       </c>
-      <c r="K6" s="243" t="s">
-        <v>504</v>
-      </c>
-      <c r="L6" s="242"/>
+      <c r="K6" s="248" t="s">
+        <v>501</v>
+      </c>
+      <c r="L6" s="247"/>
     </row>
     <row r="7" spans="1:12" ht="32" x14ac:dyDescent="0.2">
-      <c r="A7" s="245"/>
-      <c r="B7" s="246"/>
-      <c r="C7" s="245"/>
+      <c r="A7" s="244"/>
+      <c r="B7" s="245"/>
+      <c r="C7" s="244"/>
       <c r="D7" s="216" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="247"/>
-      <c r="F7" s="244"/>
-      <c r="G7" s="244"/>
-      <c r="H7" s="244"/>
-      <c r="I7" s="242"/>
-      <c r="J7" s="235"/>
-      <c r="K7" s="243"/>
-      <c r="L7" s="242"/>
+      <c r="E7" s="246"/>
+      <c r="F7" s="243"/>
+      <c r="G7" s="243"/>
+      <c r="H7" s="243"/>
+      <c r="I7" s="247"/>
+      <c r="J7" s="240"/>
+      <c r="K7" s="248"/>
+      <c r="L7" s="247"/>
     </row>
     <row r="8" spans="1:12" ht="32" x14ac:dyDescent="0.2">
-      <c r="A8" s="245"/>
-      <c r="B8" s="246"/>
-      <c r="C8" s="245"/>
+      <c r="A8" s="244"/>
+      <c r="B8" s="245"/>
+      <c r="C8" s="244"/>
       <c r="D8" s="216" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="247"/>
-      <c r="F8" s="244"/>
-      <c r="G8" s="244"/>
-      <c r="H8" s="244"/>
-      <c r="I8" s="242"/>
-      <c r="J8" s="235"/>
-      <c r="K8" s="243"/>
-      <c r="L8" s="242"/>
+      <c r="E8" s="246"/>
+      <c r="F8" s="243"/>
+      <c r="G8" s="243"/>
+      <c r="H8" s="243"/>
+      <c r="I8" s="247"/>
+      <c r="J8" s="240"/>
+      <c r="K8" s="248"/>
+      <c r="L8" s="247"/>
     </row>
     <row r="9" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="245"/>
-      <c r="B9" s="246"/>
-      <c r="C9" s="245"/>
+      <c r="A9" s="244"/>
+      <c r="B9" s="245"/>
+      <c r="C9" s="244"/>
       <c r="D9" s="139" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="247"/>
-      <c r="F9" s="244"/>
-      <c r="G9" s="244"/>
-      <c r="H9" s="244"/>
-      <c r="I9" s="242"/>
-      <c r="J9" s="235"/>
-      <c r="K9" s="243"/>
-      <c r="L9" s="242"/>
+      <c r="E9" s="246"/>
+      <c r="F9" s="243"/>
+      <c r="G9" s="243"/>
+      <c r="H9" s="243"/>
+      <c r="I9" s="247"/>
+      <c r="J9" s="240"/>
+      <c r="K9" s="248"/>
+      <c r="L9" s="247"/>
     </row>
     <row r="10" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="245"/>
-      <c r="B10" s="246"/>
-      <c r="C10" s="245"/>
+      <c r="A10" s="244"/>
+      <c r="B10" s="245"/>
+      <c r="C10" s="244"/>
       <c r="D10" s="139" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="247"/>
-      <c r="F10" s="244"/>
-      <c r="G10" s="244"/>
-      <c r="H10" s="244"/>
-      <c r="I10" s="242"/>
-      <c r="J10" s="235"/>
-      <c r="K10" s="243"/>
-      <c r="L10" s="242"/>
+      <c r="E10" s="246"/>
+      <c r="F10" s="243"/>
+      <c r="G10" s="243"/>
+      <c r="H10" s="243"/>
+      <c r="I10" s="247"/>
+      <c r="J10" s="240"/>
+      <c r="K10" s="248"/>
+      <c r="L10" s="247"/>
     </row>
     <row r="11" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="121" t="s">
@@ -17526,7 +17612,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="F11" s="124" t="s">
         <v>17</v>
@@ -17544,7 +17630,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="L11" s="107"/>
     </row>
@@ -17562,7 +17648,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="126" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -17580,7 +17666,7 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="L12" s="129" t="s">
         <v>46</v>
@@ -17600,7 +17686,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
@@ -17618,7 +17704,7 @@
         <v>29</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="L13" s="107"/>
     </row>
@@ -17636,7 +17722,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="126" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -17654,7 +17740,7 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="L14" s="129" t="s">
         <v>309</v>
@@ -17674,7 +17760,7 @@
         <v>16</v>
       </c>
       <c r="E15" s="121" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>35</v>
@@ -17819,17 +17905,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{FBE7E653-2382-46E4-9C76-9C694EDC9195}"/>
   <mergeCells count="11">
+    <mergeCell ref="L6:L10"/>
+    <mergeCell ref="K6:K10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="I6:I10"/>
+    <mergeCell ref="J6:J10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="B6:B10"/>
     <mergeCell ref="C6:C10"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="F6:F10"/>
-    <mergeCell ref="L6:L10"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="J6:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
@@ -17973,7 +18059,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="84" x14ac:dyDescent="0.2">
@@ -17990,7 +18076,7 @@
         <v>152</v>
       </c>
       <c r="E2" s="82" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>35</v>
@@ -18008,7 +18094,7 @@
         <v>37</v>
       </c>
       <c r="K2" s="107" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="L2" s="186"/>
     </row>
@@ -18046,7 +18132,7 @@
     </row>
     <row r="4" spans="1:12" ht="92.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="121" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="B4" s="35" t="s">
         <v>175</v>
@@ -18058,7 +18144,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="194" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -18196,7 +18282,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="82" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>35</v>
@@ -18214,31 +18300,31 @@
         <v>37</v>
       </c>
       <c r="K8" s="107" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="125" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="B9" s="74" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="C9" s="125" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="D9" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="212" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G9" s="127" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="H9" s="127">
         <v>1</v>
@@ -18250,31 +18336,31 @@
         <v>37</v>
       </c>
       <c r="K9" s="106" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="L9" s="129"/>
     </row>
     <row r="10" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A10" s="121" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="C10" s="121" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
       </c>
       <c r="G10" s="124" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="H10" s="133">
         <v>1</v>
@@ -18286,29 +18372,29 @@
         <v>37</v>
       </c>
       <c r="K10" s="106" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="L10" s="107"/>
     </row>
     <row r="11" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A11" s="125" t="s">
+        <v>456</v>
+      </c>
+      <c r="B11" s="74" t="s">
+        <v>457</v>
+      </c>
+      <c r="C11" s="134" t="s">
+        <v>458</v>
+      </c>
+      <c r="D11" s="154" t="s">
         <v>459</v>
-      </c>
-      <c r="B11" s="74" t="s">
-        <v>460</v>
-      </c>
-      <c r="C11" s="134" t="s">
-        <v>461</v>
-      </c>
-      <c r="D11" s="154" t="s">
-        <v>462</v>
       </c>
       <c r="E11" s="126"/>
       <c r="F11" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="H11" s="127" t="s">
         <v>19</v>
@@ -18324,13 +18410,13 @@
     </row>
     <row r="12" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="121" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="C12" s="121" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
@@ -18368,7 +18454,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="126" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
@@ -18422,19 +18508,19 @@
     </row>
     <row r="15" spans="1:12" ht="64" x14ac:dyDescent="0.2">
       <c r="A15" s="125" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="B15" s="74" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="C15" s="125" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="D15" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="126" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -18468,7 +18554,7 @@
         <v>85</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -18502,7 +18588,7 @@
         <v>92</v>
       </c>
       <c r="E17" s="80" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>35</v>
@@ -18520,7 +18606,7 @@
         <v>37</v>
       </c>
       <c r="K17" s="107" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="L17" s="129"/>
     </row>
@@ -18538,7 +18624,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -18589,7 +18675,7 @@
       </c>
       <c r="K19" s="106"/>
       <c r="L19" s="129" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="48" x14ac:dyDescent="0.2">
@@ -18606,7 +18692,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>35</v>
@@ -18630,19 +18716,19 @@
     </row>
     <row r="21" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A21" s="125" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="B21" s="74" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="C21" s="125" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="126" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -18660,10 +18746,10 @@
         <v>29</v>
       </c>
       <c r="K21" s="107" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="L21" s="192" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="48" x14ac:dyDescent="0.2">
@@ -18680,7 +18766,7 @@
         <v>333</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>35</v>
@@ -18714,7 +18800,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>35</v>
@@ -18732,7 +18818,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="106" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="L23" s="195"/>
     </row>
@@ -19215,6 +19301,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Status xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">Draft</Status>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="221af607-abea-4d5e-830c-567dcc03c0ec" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8ef391852eaca4511043a54bffd4a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="201dd8b781da46d5daa37e3355db44fe" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -19457,28 +19564,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Status xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">Draft</Status>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="221af607-abea-4d5e-830c-567dcc03c0ec" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
+    <ds:schemaRef ds:uri="221af607-abea-4d5e-830c-567dcc03c0ec"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19A23828-4FF7-4569-837D-B1B2C775409F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19495,23 +19600,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
-    <ds:schemaRef ds:uri="221af607-abea-4d5e-830c-567dcc03c0ec"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
docs: add csvw to spreadsheet and diagram
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.1.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anakonrad/Library/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{935837CE-90B2-6C41-9184-09A5A911027E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ABB04E1-A556-5B47-9055-48129A01D954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17380" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-2000" yWindow="-19520" windowWidth="38400" windowHeight="19460" firstSheet="2" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -29,12 +29,15 @@
     <sheet name="QualityCertificate" sheetId="19" r:id="rId14"/>
     <sheet name="CatalogueRecord" sheetId="10" state="hidden" r:id="rId15"/>
     <sheet name="Checksum" sheetId="11" r:id="rId16"/>
+    <sheet name="TableGroup" sheetId="21" r:id="rId17"/>
+    <sheet name="Table" sheetId="22" r:id="rId18"/>
+    <sheet name="Column" sheetId="23" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Agent!$A$1:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Catalogue!$A$1:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">DataService!$A$1:$J$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Dataset!$A$1:$J$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Dataset!$A$1:$J$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">DatasetSeries!$A$1:$L$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Distribution!$A$1:$J$23</definedName>
   </definedNames>
@@ -59,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1880" uniqueCount="688">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2034" uniqueCount="738">
   <si>
     <t>Property label</t>
   </si>
@@ -2743,12 +2746,201 @@
 If a limit is known, provide both dcat:startDate and dcat:endDate.</t>
     </r>
   </si>
+  <si>
+    <t>variables</t>
+  </si>
+  <si>
+    <t>healthdcatap:hasVariables</t>
+  </si>
+  <si>
+    <t>Links the Dataset to a CSVW TableGroup that provides a machine-readable description of the data variables.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+      </rPr>
+      <t>Note</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+      </rPr>
+      <t>: The variables  have been added to the metadata model version 2.1 for testing purposes. For now it is not yet planned to be added to the national catalogue's front end.
+Use this property to link a structured dataset to a CSVW TableGroup that documents its data variables, columns, or fields in a machine-readable way.</t>
+    </r>
+  </si>
+  <si>
+    <t>table</t>
+  </si>
+  <si>
+    <t>A table is a single CSV file within a CSVW Table Group.</t>
+  </si>
+  <si>
+    <t>csvw:table</t>
+  </si>
+  <si>
+    <t>Used to associate one or more tables with a table group. It holds all variable dictionary entries, using columns describing each variable.</t>
+  </si>
+  <si>
+    <t>csvw:Table</t>
+  </si>
+  <si>
+    <t>Value: table 1</t>
+  </si>
+  <si>
+    <t>Value: table 2</t>
+  </si>
+  <si>
+    <t>Add more columns if you need to describe additional instances of csvw:TableGroup</t>
+  </si>
+  <si>
+    <t>csvw:TableGroup</t>
+  </si>
+  <si>
+    <t>fill in in 'TableGroup' tab</t>
+  </si>
+  <si>
+    <t>fill in in 'TableGroup'  tab</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>column</t>
+  </si>
+  <si>
+    <t>The URL of the CSV file to which this table refers.</t>
+  </si>
+  <si>
+    <t>Table title.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A keyword or tag describing the table.	</t>
+  </si>
+  <si>
+    <t>Variable (column) defines metadata about one field in the CSV file.</t>
+  </si>
+  <si>
+    <t>IRI</t>
+  </si>
+  <si>
+    <t>csvw:url</t>
+  </si>
+  <si>
+    <t>csvw:title</t>
+  </si>
+  <si>
+    <t>csvw:column</t>
+  </si>
+  <si>
+    <t>The URL should be a valid IRI and should point to the CSV file (synthetic, anonymized representation of the real data) for this table.</t>
+  </si>
+  <si>
+    <t>Used to provide a human-readable title for the table. Can appear in multiple languages.</t>
+  </si>
+  <si>
+    <t>Provides a set of keywords to support search and discovery of the table.</t>
+  </si>
+  <si>
+    <t>Each variable (column) node defines characteristics such as name, title, datatype, etc., for one column of the CSV. Should be either a blank node or IRI referring to a csvw:Column.</t>
+  </si>
+  <si>
+    <t>csvw:Column</t>
+  </si>
+  <si>
+    <t>Add more columns if you need to describe additional instances of csvw:Table</t>
+  </si>
+  <si>
+    <t>datatype</t>
+  </si>
+  <si>
+    <t>property URL</t>
+  </si>
+  <si>
+    <t>A Technical name given to the Variable as it appears in the CSV file.</t>
+  </si>
+  <si>
+    <t>A Human-readable name given to the Variable.</t>
+  </si>
+  <si>
+    <t>Variable description.</t>
+  </si>
+  <si>
+    <t>Specifies the expected datatype of the values in the column.</t>
+  </si>
+  <si>
+    <t>A URI template used to define the RDF predicate associated with the values in the column, relative to each row.</t>
+  </si>
+  <si>
+    <t>csvw:name</t>
+  </si>
+  <si>
+    <t>csvw:datatype</t>
+  </si>
+  <si>
+    <t>csvw:propetyUrl</t>
+  </si>
+  <si>
+    <t>Technical variable name required to match a column header in the CSV file (synthetic, anonymized representation of the real data), can appear in multiple languages.</t>
+  </si>
+  <si>
+    <t>Human-readable title(s) for the column. May be multilingual.</t>
+  </si>
+  <si>
+    <t>Used to provide human-readable information about the variable (column). Can appear in multiple languages. This is especially helpful for variable documentation.</t>
+  </si>
+  <si>
+    <t>https://w3c.github.io/csvw/metadata/#datatypes</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Should match the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>label</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> of one of the CSVW types as defined in the Built-in datatypes from XML Schema. https://w3c.github.io/csvw/metadata/#datatypes Example: string, integer, boolean …</t>
+    </r>
+  </si>
+  <si>
+    <t>The propertyUrl may point to standard, controlled vocabularies, or ontologies that define the semantic meaning of the column. For example: csvw:propertyUrl &lt;http://publications.europa.eu/resource/authority/country&gt; For advanced usage, refer to the official specification: https://www.w3.org/TR/tabular-metadata/#propertyurl</t>
+  </si>
+  <si>
+    <t>Value: column 1</t>
+  </si>
+  <si>
+    <t>Value: column 2</t>
+  </si>
+  <si>
+    <t>xsd:anyURI</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="56" x14ac:knownFonts="1">
+  <fonts count="57" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3106,6 +3298,13 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="14">
     <fill>
@@ -3209,7 +3408,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="250">
+  <cellXfs count="258">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3939,13 +4138,67 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="191">
+  <dxfs count="263">
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -3968,6 +4221,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3978,6 +4251,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -3988,6 +4291,176 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -3998,6 +4471,26 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4008,6 +4501,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -4102,7 +4615,17 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor theme="2"/>
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4118,6 +4641,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -4128,6 +4671,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -4138,6 +4721,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4152,6 +4755,16 @@
       </font>
       <fill>
         <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
           <bgColor theme="4" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
@@ -4188,6 +4801,46 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4198,6 +4851,26 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4208,6 +4881,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -4218,6 +4911,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -4228,6 +4961,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4238,6 +4981,206 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -4248,6 +5191,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -4258,6 +5211,26 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4268,6 +5241,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -4278,6 +5261,46 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4288,6 +5311,26 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4298,6 +5341,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -4318,121 +5371,11 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
     </dxf>
@@ -7659,35 +8602,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="104" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="176" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="103" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="175" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="174" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="173" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="172" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="99" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="171" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="170" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="169" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="168" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8349,71 +9292,71 @@
     <sortCondition ref="A2:A3"/>
   </sortState>
   <conditionalFormatting sqref="A41:B42">
-    <cfRule type="cellIs" dxfId="95" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="167" priority="11" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="166" priority="12" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="165" priority="13" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="92" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="164" priority="14" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D40:E42">
-    <cfRule type="cellIs" dxfId="91" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="163" priority="15" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="162" priority="16" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="161" priority="17" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="160" priority="18" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F52">
-    <cfRule type="cellIs" dxfId="87" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="159" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="86" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="158" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="157" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="156" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="155" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="82" priority="19" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="154" priority="19" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="153" priority="20" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F52">
-    <cfRule type="cellIs" dxfId="80" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="152" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="151" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="150" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="77" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="149" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8587,35 +9530,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="76" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="148" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="75" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="147" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="146" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="145" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="144" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="71" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="143" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="142" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="141" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="140" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8772,35 +9715,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="67" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="139" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="66" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="138" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="65" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="137" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="136" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="135" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="62" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="134" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="133" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="132" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="59" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="131" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8957,35 +9900,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="58" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="130" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="57" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="129" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="128" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="127" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="126" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="125" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="124" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="123" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="122" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9597,97 +10540,97 @@
     <sortCondition ref="A2:A10"/>
   </sortState>
   <conditionalFormatting sqref="A27:B28">
-    <cfRule type="cellIs" dxfId="49" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="121" priority="41" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="120" priority="42" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="119" priority="43" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="118" priority="44" operator="equal">
       <formula>"Conditional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="43" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="42" operator="equal">
-      <formula>"Recommended"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D26:E28">
-    <cfRule type="cellIs" dxfId="45" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="117" priority="45" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="116" priority="46" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="47" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="114" priority="48" operator="equal">
       <formula>"Conditional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="47" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="46" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="45" operator="equal">
-      <formula>"Optional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8">
-    <cfRule type="cellIs" dxfId="41" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="51" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="112" priority="52" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="111" priority="53" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="110" priority="54" operator="equal">
       <formula>"Conditional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="51" operator="equal">
-      <formula>"Optional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="52" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="53" operator="equal">
-      <formula>"Mandatory"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F7 E8">
-    <cfRule type="cellIs" dxfId="37" priority="40" operator="equal">
+    <cfRule type="cellIs" dxfId="109" priority="40" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9:F38">
-    <cfRule type="cellIs" dxfId="36" priority="38" operator="equal">
+    <cfRule type="cellIs" dxfId="108" priority="33" operator="equal">
+      <formula>"Not added"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="107" priority="36" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="106" priority="37" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="105" priority="38" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="39" operator="equal">
+    <cfRule type="cellIs" dxfId="104" priority="39" operator="equal">
       <formula>"Conditional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="37" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="36" operator="equal">
-      <formula>"Optional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="33" operator="equal">
-      <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H11">
-    <cfRule type="cellIs" dxfId="31" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="103" priority="9" operator="greaterThan">
+      <formula>"reviewd"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="102" priority="10" operator="equal">
       <formula>"needs review"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="9" operator="greaterThan">
-      <formula>"reviewd"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14:H27 H36:H38">
-    <cfRule type="cellIs" dxfId="29" priority="49" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="101" priority="49" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="100" priority="50" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F7">
-    <cfRule type="cellIs" dxfId="27" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="15" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="98" priority="16" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="97" priority="17" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="96" priority="18" operator="equal">
       <formula>"Conditional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="17" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="16" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="15" operator="equal">
-      <formula>"Optional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -10330,89 +11273,89 @@
     <sortCondition ref="A2:A3"/>
   </sortState>
   <conditionalFormatting sqref="A41:B42">
-    <cfRule type="cellIs" dxfId="23" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="95" priority="21" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="94" priority="22" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="93" priority="23" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="92" priority="24" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D40:E42">
-    <cfRule type="cellIs" dxfId="19" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="91" priority="25" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="26" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="89" priority="27" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="88" priority="28" operator="equal">
       <formula>"Conditional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="27" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="26" operator="equal">
-      <formula>"Recommended"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E3">
-    <cfRule type="cellIs" dxfId="15" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="87" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="86" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F52">
-    <cfRule type="cellIs" dxfId="10" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="10" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G3">
-    <cfRule type="cellIs" dxfId="9" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="81" priority="16" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="17" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="79" priority="18" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="19" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="5" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="29" operator="greaterThan">
+      <formula>"reviewd"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="76" priority="30" operator="equal">
       <formula>"needs review"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="29" operator="greaterThan">
-      <formula>"reviewd"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F52">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="1" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="74" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="73" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="72" priority="4" operator="equal">
       <formula>"Conditional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"Optional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -10435,6 +11378,2251 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" location="d4e2129" xr:uid="{611386D8-2287-4730-A668-74EE9D69BC9E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67277BAE-CBA0-C04C-8D1F-19B83637B929}">
+  <sheetPr>
+    <tabColor theme="5" tint="0.79998168889431442"/>
+  </sheetPr>
+  <dimension ref="A1:N51"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.83203125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="28.5" style="9" customWidth="1"/>
+    <col min="3" max="4" width="17.83203125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="27.83203125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="17.83203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="26.5" style="2" customWidth="1"/>
+    <col min="8" max="10" width="17.83203125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" style="2" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="17.5" style="2" customWidth="1"/>
+    <col min="13" max="13" width="19.5" style="2" customWidth="1"/>
+    <col min="14" max="14" width="33.1640625" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="9.1640625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="89" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="89" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="89" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="91" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="89" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="89" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="89" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="89" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="90" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="90" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="219" t="s">
+        <v>697</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>698</v>
+      </c>
+      <c r="N1" s="233" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="64" x14ac:dyDescent="0.2">
+      <c r="A2" s="44" t="s">
+        <v>692</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>693</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>694</v>
+      </c>
+      <c r="D2" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="197" t="s">
+        <v>695</v>
+      </c>
+      <c r="F2" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" s="257" t="s">
+        <v>696</v>
+      </c>
+      <c r="H2" s="47" t="s">
+        <v>52</v>
+      </c>
+      <c r="I2" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="47" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A3" s="13"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A4" s="13"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="4"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A5" s="13"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A6" s="13"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A7" s="13"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A8" s="13"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="3"/>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" s="13"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" s="13"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" s="13"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12" s="13"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13" s="13"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" s="13"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="13"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A15" s="13"/>
+      <c r="B15" s="11"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A16" s="13"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="20"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="13"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="13"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="20"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="13"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="13"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" s="13"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="6"/>
+      <c r="H21" s="20"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" s="13"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="20"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" s="13"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="4"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="13"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="4"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" s="13"/>
+      <c r="B25" s="8"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="13"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="13"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="4"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" s="13"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="13"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="256"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A28" s="13"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="4"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" s="13"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="4"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="13"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="4"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" s="13"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="4"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A32" s="13"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="4"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="13"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="4"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="13"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="4"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="13"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="4"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" s="13"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="4"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" s="13"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="4"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" s="13"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="4"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" s="13"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="11"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="4"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" s="13"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" s="13"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="3"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" s="13"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="3"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" s="13"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" s="13"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="12"/>
+      <c r="H44" s="3"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" s="13"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="3"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" s="13"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="3"/>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" s="13"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" s="13"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" s="13"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="8"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="4"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" s="13"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="4"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="13"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="4"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A40:B41 F1:F51">
+    <cfRule type="cellIs" dxfId="71" priority="15" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="70" priority="16" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="69" priority="17" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="68" priority="18" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D39:E41">
+    <cfRule type="cellIs" dxfId="67" priority="19" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="66" priority="20" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="65" priority="21" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="64" priority="22" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2">
+    <cfRule type="cellIs" dxfId="63" priority="5" operator="equal">
+      <formula>"Not added"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="62" priority="6" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="61" priority="7" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="60" priority="8" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="59" priority="9" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F51">
+    <cfRule type="cellIs" dxfId="58" priority="10" operator="equal">
+      <formula>"Not added"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2">
+    <cfRule type="cellIs" dxfId="57" priority="11" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="56" priority="12" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="55" priority="13" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="54" priority="14" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H8 H10:H14 H16:H24 H26:H40 H49:H51">
+    <cfRule type="cellIs" dxfId="53" priority="23" operator="greaterThan">
+      <formula>"reviewd"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="52" priority="24" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1:I1">
+    <cfRule type="cellIs" dxfId="51" priority="1" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="50" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="49" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="48" priority="4" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="6">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2 J1" xr:uid="{FC70BEFA-A7EE-C949-9135-F0A5F5075E51}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F51" xr:uid="{EBB64232-5E14-5846-9C7F-2F6379FF2CEF}">
+      <formula1>"Mandatory, Recommended, Optional, Conditional, Not added"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H49:H51 H26:H40 H10:H14 H16:H24 H3:H8" xr:uid="{AC2185B6-FA30-CF48-8407-4F028DEFDAFD}">
+      <formula1>"0..n, 0..1, 1, 1..n"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F2" xr:uid="{FD6D9053-0604-8541-BE23-D9FA05456B54}">
+      <formula1>"Mandatory, Recommended, Optional, Conditional"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{F80C0C95-06A2-474A-94CF-5BFD7EFAEBCE}">
+      <formula1>"DCAT-AP v3, HealthDCAT-AP, DCAT-AP NL, HRI v1"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576" xr:uid="{8E8D2392-D891-8947-BEF6-AD37A6D6DF98}">
+      <formula1>"Identical to v1, Adapted from v1, new"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7708DCAE-0CF1-3848-BA07-512C5955A6D7}">
+  <sheetPr>
+    <tabColor theme="5" tint="0.79998168889431442"/>
+  </sheetPr>
+  <dimension ref="A1:N52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.83203125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="28.5" style="9" customWidth="1"/>
+    <col min="3" max="4" width="17.83203125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="27.83203125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="17.83203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="26.5" style="2" customWidth="1"/>
+    <col min="8" max="10" width="17.83203125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" style="2" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="17.5" style="2" customWidth="1"/>
+    <col min="13" max="13" width="19.5" style="2" customWidth="1"/>
+    <col min="14" max="14" width="33.1640625" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="9.1640625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="89" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="89" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="89" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="91" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="89" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="89" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="89" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="89" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="90" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="90" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="219" t="s">
+        <v>697</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>698</v>
+      </c>
+      <c r="N1" s="233" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="80" x14ac:dyDescent="0.2">
+      <c r="A2" s="44" t="s">
+        <v>703</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>705</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>710</v>
+      </c>
+      <c r="D2" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="197" t="s">
+        <v>713</v>
+      </c>
+      <c r="F2" s="46" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="H2" s="204" t="s">
+        <v>81</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="47" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="48" x14ac:dyDescent="0.2">
+      <c r="A3" s="44" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" s="250" t="s">
+        <v>706</v>
+      </c>
+      <c r="C3" s="251" t="s">
+        <v>133</v>
+      </c>
+      <c r="D3" s="252" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="253" t="s">
+        <v>714</v>
+      </c>
+      <c r="F3" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="254" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="47" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="42" x14ac:dyDescent="0.2">
+      <c r="A4" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>707</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="D4" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="96" x14ac:dyDescent="0.2">
+      <c r="A5" s="13" t="s">
+        <v>704</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>708</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>712</v>
+      </c>
+      <c r="D5" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>716</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="255" t="s">
+        <v>717</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A6" s="13"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A7" s="13"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A8" s="13"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" s="13"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="3"/>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" s="13"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" s="13"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12" s="13"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13" s="13"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" s="13"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A15" s="13"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="13"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A16" s="13"/>
+      <c r="B16" s="11"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="13"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="20"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="13"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="13"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="20"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="13"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="13"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="13"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="6"/>
+      <c r="H22" s="20"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="13"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="20"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="13"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="4"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" s="13"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="4"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="13"/>
+      <c r="B26" s="8"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="13"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="13"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="4"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="13"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="13"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="4"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" s="13"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="4"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="13"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="4"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="13"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="4"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" s="13"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="4"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="13"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="4"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="13"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="4"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="13"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="4"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" s="13"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="4"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" s="13"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="4"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" s="13"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="4"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" s="13"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="11"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="4"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" s="13"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="4"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" s="13"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" s="13"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="3"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" s="13"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="3"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" s="13"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" s="13"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="3"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" s="13"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" s="13"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="3"/>
+      <c r="H47" s="3"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" s="13"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" s="13"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" s="13"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="4"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="13"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="4"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" s="13"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="13"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="4"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A41:B42 F1:F52">
+    <cfRule type="cellIs" dxfId="47" priority="15" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="46" priority="16" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="17" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="44" priority="18" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D40:E42">
+    <cfRule type="cellIs" dxfId="43" priority="19" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="20" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="41" priority="21" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="22" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E3">
+    <cfRule type="cellIs" dxfId="39" priority="5" operator="equal">
+      <formula>"Not added"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="6" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="7" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="36" priority="8" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="35" priority="9" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F52">
+    <cfRule type="cellIs" dxfId="34" priority="10" operator="equal">
+      <formula>"Not added"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H3">
+    <cfRule type="cellIs" dxfId="33" priority="11" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="12" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="31" priority="13" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="14" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H6:H9 H11:H15 H17:H25 H27:H41 H50:H52">
+    <cfRule type="cellIs" dxfId="29" priority="23" operator="greaterThan">
+      <formula>"reviewd"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="24" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1:I1">
+    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="4" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{B788B1F1-4C8F-5C42-923C-153A35CEEA5C}">
+      <formula1>"DCAT-AP v3, HealthDCAT-AP, DCAT-AP NL, HRI v1"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F3" xr:uid="{5D979C31-746D-D040-A470-B87E1D05BB97}">
+      <formula1>"Mandatory, Recommended, Optional, Conditional"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H50:H52 H27:H41 H11:H15 H17:H25 H6:H9" xr:uid="{FA77196E-8222-E547-9612-265E91F8A772}">
+      <formula1>"0..n, 0..1, 1, 1..n"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F52" xr:uid="{88A055E7-7E23-C94D-B9C0-687FEBD8E3B9}">
+      <formula1>"Mandatory, Recommended, Optional, Conditional, Not added"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3 J1" xr:uid="{E03EA4F6-9910-094B-B7B5-9532E18C5064}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4:I1048576" xr:uid="{1BCF2E28-5DEB-B444-9E3C-F41046936230}">
+      <formula1>"Identical to v1, Adapted from v1, new"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00C65873-9AF7-7944-82C8-6D469506ACC7}">
+  <sheetPr>
+    <tabColor theme="5" tint="0.79998168889431442"/>
+  </sheetPr>
+  <dimension ref="A1:N52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.83203125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="28.5" style="9" customWidth="1"/>
+    <col min="3" max="4" width="17.83203125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="27.83203125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="17.83203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="26.5" style="2" customWidth="1"/>
+    <col min="8" max="10" width="17.83203125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" style="2" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="17.5" style="2" customWidth="1"/>
+    <col min="13" max="13" width="19.5" style="2" customWidth="1"/>
+    <col min="14" max="14" width="33.1640625" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="9.1640625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="89" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="89" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="89" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="91" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="89" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="89" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="89" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="89" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="90" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="90" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="219" t="s">
+        <v>735</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>736</v>
+      </c>
+      <c r="N1" s="233" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="80" x14ac:dyDescent="0.2">
+      <c r="A2" s="44" t="s">
+        <v>375</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>721</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>726</v>
+      </c>
+      <c r="D2" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="197" t="s">
+        <v>729</v>
+      </c>
+      <c r="F2" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" s="204" t="s">
+        <v>52</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="47" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+      <c r="A3" s="44" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" s="250" t="s">
+        <v>722</v>
+      </c>
+      <c r="C3" s="251" t="s">
+        <v>711</v>
+      </c>
+      <c r="D3" s="252" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="253" t="s">
+        <v>730</v>
+      </c>
+      <c r="F3" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="254" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="47" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="84" x14ac:dyDescent="0.2">
+      <c r="A4" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>723</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D4" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>731</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="112" x14ac:dyDescent="0.2">
+      <c r="A5" s="13" t="s">
+        <v>719</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>724</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>727</v>
+      </c>
+      <c r="D5" s="78" t="s">
+        <v>732</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>733</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5" s="3">
+        <v>1</v>
+      </c>
+      <c r="I5" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="154" x14ac:dyDescent="0.2">
+      <c r="A6" s="13" t="s">
+        <v>720</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>725</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>728</v>
+      </c>
+      <c r="D6" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>734</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>709</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A7" s="13"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A8" s="13"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" s="13"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="3"/>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" s="13"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" s="13"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12" s="13"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13" s="13"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" s="13"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A15" s="13"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="13"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A16" s="13"/>
+      <c r="B16" s="11"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="13"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="20"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="13"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="13"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="20"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="13"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="13"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="13"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="6"/>
+      <c r="H22" s="20"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="13"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="20"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="13"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="4"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" s="13"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="4"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="13"/>
+      <c r="B26" s="8"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="13"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="13"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="4"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="13"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="13"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="4"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" s="13"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="4"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="13"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="4"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="13"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="4"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" s="13"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="4"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="13"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="4"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="13"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="4"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="13"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="4"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" s="13"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="4"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" s="13"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="4"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" s="13"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="4"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" s="13"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="11"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="4"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" s="13"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="4"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" s="13"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" s="13"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="3"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" s="13"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="3"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" s="13"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" s="13"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="3"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" s="13"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" s="13"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="3"/>
+      <c r="H47" s="3"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" s="13"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" s="13"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" s="13"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="4"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="13"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="4"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" s="13"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="13"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="4"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A41:B42 F1:F52">
+    <cfRule type="cellIs" dxfId="23" priority="15" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="16" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="17" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="18" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D40:E42">
+    <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="20" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="17" priority="21" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="22" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E3">
+    <cfRule type="cellIs" dxfId="15" priority="5" operator="equal">
+      <formula>"Not added"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="6" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="7" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="8" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="11" priority="9" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F52">
+    <cfRule type="cellIs" dxfId="10" priority="10" operator="equal">
+      <formula>"Not added"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H3">
+    <cfRule type="cellIs" dxfId="9" priority="11" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="12" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="13" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="14" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H6:H9 H11:H15 H17:H25 H27:H41 H50:H52">
+    <cfRule type="cellIs" dxfId="5" priority="23" operator="greaterThan">
+      <formula>"reviewd"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="24" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1:I1">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4:I1048576" xr:uid="{B293199C-D0AA-4E45-AB74-A455D76C8259}">
+      <formula1>"Identical to v1, Adapted from v1, new"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3 J1" xr:uid="{A8C9190A-EEC6-3645-ABEC-B4A9A5787002}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F52" xr:uid="{98A6158D-25B4-3742-8B36-5DF546930EFF}">
+      <formula1>"Mandatory, Recommended, Optional, Conditional, Not added"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H50:H52 H27:H41 H11:H15 H17:H25 H6:H9" xr:uid="{AF68AF06-9542-854E-ABFA-F6B15E8FC7AA}">
+      <formula1>"0..n, 0..1, 1, 1..n"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F3" xr:uid="{98F91931-2B9A-F443-9CD5-804BEA4B4484}">
+      <formula1>"Mandatory, Recommended, Optional, Conditional"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{8F58434A-654C-E049-8544-7737E87C06AF}">
+      <formula1>"DCAT-AP v3, HealthDCAT-AP, DCAT-AP NL, HRI v1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="D5" r:id="rId1" location="datatypes" xr:uid="{BD93A683-D377-FD4E-B01D-82A045F4E583}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11674,71 +14862,71 @@
     <mergeCell ref="F8:F12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
-    <cfRule type="cellIs" dxfId="190" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="262" priority="16" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F13:F56">
-    <cfRule type="cellIs" dxfId="189" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="261" priority="26" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="188" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="260" priority="29" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="187" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="259" priority="30" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="186" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="258" priority="31" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="185" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="257" priority="32" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H8 H13:H56">
-    <cfRule type="cellIs" dxfId="184" priority="17" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="256" priority="17" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="183" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="255" priority="18" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F8">
-    <cfRule type="cellIs" dxfId="182" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="254" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="181" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="253" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="180" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="252" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="179" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="251" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J8 J13:J56">
-    <cfRule type="containsText" dxfId="178" priority="13" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="250" priority="13" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="177" priority="14" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="249" priority="14" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="176" priority="15" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="248" priority="15" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1">
-    <cfRule type="cellIs" dxfId="175" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="247" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="174" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="246" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="173" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="245" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="172" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="244" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11788,7 +14976,7 @@
     <tabColor rgb="FFC00000"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.5" style="41" bestFit="1" customWidth="1"/>
@@ -13713,134 +16901,176 @@
       <c r="M52" s="129"/>
       <c r="N52" s="129"/>
     </row>
-    <row r="53" spans="1:14" ht="32" x14ac:dyDescent="0.2">
-      <c r="A53" s="121" t="s">
+    <row r="53" spans="1:14" ht="80" x14ac:dyDescent="0.2">
+      <c r="A53" s="125" t="s">
+        <v>688</v>
+      </c>
+      <c r="B53" s="74" t="s">
+        <v>690</v>
+      </c>
+      <c r="C53" s="125" t="s">
+        <v>689</v>
+      </c>
+      <c r="D53" s="217" t="s">
+        <v>16</v>
+      </c>
+      <c r="E53" s="83" t="s">
+        <v>691</v>
+      </c>
+      <c r="F53" s="127" t="s">
+        <v>17</v>
+      </c>
+      <c r="G53" s="128" t="s">
+        <v>700</v>
+      </c>
+      <c r="H53" s="127" t="s">
+        <v>19</v>
+      </c>
+      <c r="I53" s="129" t="s">
+        <v>20</v>
+      </c>
+      <c r="J53" s="129" t="s">
+        <v>66</v>
+      </c>
+      <c r="K53" s="130"/>
+      <c r="L53" s="129" t="s">
+        <v>701</v>
+      </c>
+      <c r="M53" s="129" t="s">
+        <v>702</v>
+      </c>
+      <c r="N53" s="129" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+      <c r="A54" s="121" t="s">
         <v>341</v>
       </c>
-      <c r="B53" s="35" t="s">
+      <c r="B54" s="35" t="s">
         <v>342</v>
       </c>
-      <c r="C53" s="121" t="s">
+      <c r="C54" s="121" t="s">
         <v>343</v>
       </c>
-      <c r="D53" s="132" t="s">
+      <c r="D54" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="E53" s="132" t="s">
+      <c r="E54" s="132" t="s">
         <v>344</v>
       </c>
-      <c r="F53" s="124" t="s">
+      <c r="F54" s="124" t="s">
         <v>17</v>
       </c>
-      <c r="G53" s="124" t="s">
+      <c r="G54" s="124" t="s">
         <v>58</v>
       </c>
-      <c r="H53" s="124" t="s">
+      <c r="H54" s="124" t="s">
         <v>81</v>
       </c>
-      <c r="I53" s="107" t="s">
+      <c r="I54" s="107" t="s">
         <v>104</v>
       </c>
-      <c r="J53" s="107" t="s">
+      <c r="J54" s="107" t="s">
         <v>37</v>
       </c>
-      <c r="K53" s="106" t="s">
+      <c r="K54" s="106" t="s">
         <v>144</v>
       </c>
-      <c r="L53" s="107"/>
-      <c r="M53" s="107"/>
-      <c r="N53" s="107"/>
-    </row>
-    <row r="54" spans="1:14" ht="32" x14ac:dyDescent="0.2">
-      <c r="A54" s="125" t="s">
+      <c r="L54" s="107"/>
+      <c r="M54" s="107"/>
+      <c r="N54" s="107"/>
+    </row>
+    <row r="55" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+      <c r="A55" s="125" t="s">
         <v>345</v>
       </c>
-      <c r="B54" s="74" t="s">
+      <c r="B55" s="74" t="s">
         <v>346</v>
       </c>
-      <c r="C54" s="125" t="s">
+      <c r="C55" s="125" t="s">
         <v>347</v>
       </c>
-      <c r="D54" s="126" t="s">
+      <c r="D55" s="126" t="s">
         <v>16</v>
       </c>
-      <c r="E54" s="74" t="s">
+      <c r="E55" s="74" t="s">
         <v>348</v>
       </c>
-      <c r="F54" s="127" t="s">
+      <c r="F55" s="127" t="s">
         <v>17</v>
       </c>
-      <c r="G54" s="127" t="s">
+      <c r="G55" s="127" t="s">
         <v>58</v>
       </c>
-      <c r="H54" s="127" t="s">
+      <c r="H55" s="127" t="s">
         <v>19</v>
       </c>
-      <c r="I54" s="129" t="s">
+      <c r="I55" s="129" t="s">
         <v>20</v>
       </c>
-      <c r="J54" s="129" t="s">
+      <c r="J55" s="129" t="s">
         <v>29</v>
       </c>
-      <c r="K54" s="130" t="s">
+      <c r="K55" s="130" t="s">
         <v>145</v>
       </c>
-      <c r="L54" s="129"/>
-      <c r="M54" s="129"/>
-      <c r="N54" s="129"/>
-    </row>
-    <row r="55" spans="1:14" ht="84.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="121" t="s">
+      <c r="L55" s="129"/>
+      <c r="M55" s="129"/>
+      <c r="N55" s="129"/>
+    </row>
+    <row r="56" spans="1:14" ht="84.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="121" t="s">
         <v>349</v>
       </c>
-      <c r="B55" s="35" t="s">
+      <c r="B56" s="35" t="s">
         <v>350</v>
       </c>
-      <c r="C55" s="121" t="s">
+      <c r="C56" s="121" t="s">
         <v>351</v>
       </c>
-      <c r="D55" s="132" t="s">
+      <c r="D56" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="E55" s="132"/>
-      <c r="F55" s="124" t="s">
+      <c r="E56" s="132"/>
+      <c r="F56" s="124" t="s">
         <v>17</v>
       </c>
-      <c r="G55" s="124" t="s">
+      <c r="G56" s="124" t="s">
         <v>352</v>
       </c>
-      <c r="H55" s="124" t="s">
+      <c r="H56" s="124" t="s">
         <v>19</v>
       </c>
-      <c r="I55" s="107" t="s">
+      <c r="I56" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="J55" s="107" t="s">
+      <c r="J56" s="107" t="s">
         <v>29</v>
       </c>
-      <c r="K55" s="106"/>
-      <c r="L55" s="107"/>
-      <c r="M55" s="107"/>
-      <c r="N55" s="107"/>
-    </row>
-    <row r="56" spans="1:14" s="118" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="145"/>
-      <c r="B56" s="146"/>
-      <c r="C56" s="145"/>
-      <c r="D56" s="147"/>
-      <c r="E56" s="147"/>
-      <c r="F56" s="148"/>
-      <c r="G56" s="148"/>
-      <c r="H56" s="148"/>
-      <c r="I56" s="149"/>
-      <c r="J56" s="149"/>
-      <c r="K56" s="150"/>
-      <c r="L56" s="149"/>
+      <c r="K56" s="106"/>
+      <c r="L56" s="107"/>
+      <c r="M56" s="107"/>
+      <c r="N56" s="107"/>
+    </row>
+    <row r="57" spans="1:14" s="118" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="145"/>
+      <c r="B57" s="146"/>
+      <c r="C57" s="145"/>
+      <c r="D57" s="147"/>
+      <c r="E57" s="147"/>
+      <c r="F57" s="148"/>
+      <c r="G57" s="148"/>
+      <c r="H57" s="148"/>
+      <c r="I57" s="149"/>
+      <c r="J57" s="149"/>
+      <c r="K57" s="150"/>
+      <c r="L57" s="149"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J56" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J56">
-    <sortCondition ref="A2:A56"/>
+  <autoFilter ref="A1:J57" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J57">
+    <sortCondition ref="A2:A57"/>
   </sortState>
   <mergeCells count="11">
     <mergeCell ref="L15:L19"/>
@@ -13855,55 +17085,55 @@
     <mergeCell ref="F15:F19"/>
     <mergeCell ref="E15:E19"/>
   </mergeCells>
-  <conditionalFormatting sqref="F2:F15 F20:F56">
-    <cfRule type="cellIs" dxfId="171" priority="8" operator="equal">
+  <conditionalFormatting sqref="F2:F15 F20:F57">
+    <cfRule type="cellIs" dxfId="243" priority="8" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H15 H20:H56">
-    <cfRule type="cellIs" dxfId="170" priority="17" operator="greaterThan">
+  <conditionalFormatting sqref="H2:H15 H20:H57">
+    <cfRule type="cellIs" dxfId="242" priority="17" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="169" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="241" priority="18" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:I1 F1:F15 F20:F56">
-    <cfRule type="cellIs" dxfId="168" priority="19" operator="equal">
+  <conditionalFormatting sqref="H1:I1 F1:F15 F20:F57">
+    <cfRule type="cellIs" dxfId="240" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="167" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="239" priority="20" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="166" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="238" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="165" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="237" priority="22" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J15 J20:J56">
-    <cfRule type="containsText" dxfId="164" priority="5" operator="containsText" text="Health and NL">
+  <conditionalFormatting sqref="J2:J15 J20:J57">
+    <cfRule type="containsText" dxfId="236" priority="5" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="163" priority="6" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="235" priority="6" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="162" priority="7" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="234" priority="7" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1">
-    <cfRule type="cellIs" dxfId="161" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="233" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="160" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="232" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="159" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="231" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="158" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="230" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13911,17 +17141,17 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1" xr:uid="{7D4DA44D-79A1-46A0-A570-1C5C4461BB54}">
       <formula1>"Mandatory, Recommended, Optional, Conditional"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H50:H56 H15 H30:H41 H20:H28 H2:H13" xr:uid="{9762E750-ADF5-4984-93BF-D8ED80389E8E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H50:H57 H15 H30:H41 H20:H28 H2:H13" xr:uid="{9762E750-ADF5-4984-93BF-D8ED80389E8E}">
       <formula1>"0..n, 0..1, 1, 1..n"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1 J51 J55:J56" xr:uid="{D74C1692-73CE-477E-BF57-68FEA17E3FE5}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J52:J54 J56 J20:J50 J2:J15" xr:uid="{B80CEB2B-1BEF-4952-992A-5359B9DD2C11}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1 J51 J56:J57" xr:uid="{D74C1692-73CE-477E-BF57-68FEA17E3FE5}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J52:J55 J57 J20:J50 J2:J15" xr:uid="{B80CEB2B-1BEF-4952-992A-5359B9DD2C11}">
       <formula1>"DCAT-AP v3, HealthDCAT-AP, DCAT-AP NL, HRI v1, Health and NL"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I20:I1048576 K57:K1048576 I2:I15" xr:uid="{96DDE4B1-378F-48ED-B590-490B6967CC12}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I20:I1048576 K58:K1048576 I2:I15" xr:uid="{96DDE4B1-378F-48ED-B590-490B6967CC12}">
       <formula1>"Identical to v1, Adapted from v1, new"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F20:F56 F2:F15" xr:uid="{584B70CE-0B19-4CA2-8DA1-B7818B2A385E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F20:F57 F2:F15" xr:uid="{584B70CE-0B19-4CA2-8DA1-B7818B2A385E}">
       <formula1>"Mandatory, Recommended, Optional, Conditional, Not added"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Input value in the Agent tab user Dataset (Publisher) column" sqref="A38" xr:uid="{2B8CEDBE-F99A-4484-AF52-1F52713C546E}"/>
@@ -13930,7 +17160,7 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please use the tab Relationship to fill out the values" sqref="A41" xr:uid="{EDE28D90-6B7E-4FAD-BDD1-0DAA34F97E0D}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please use tab QualityCertificate tab to fill out values" sqref="A42" xr:uid="{11657F8E-91CA-4E92-B36A-B639678885AA}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please use Attribution tab to fill out values" sqref="A40" xr:uid="{E26EB923-68C6-4995-974E-0BC6C7BE1967}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J57:J1048576" xr:uid="{1E5E2E20-49B0-42CC-AEB2-F591D86C2104}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J58:J1048576" xr:uid="{1E5E2E20-49B0-42CC-AEB2-F591D86C2104}">
       <formula1>"DCAT-AP v3, HealthDCAT-AP, DCAT-AP NL, HRI v1"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please use PeriodOfTime tab to fill out values" sqref="A48" xr:uid="{3B59EB1E-056E-4C6F-87C4-7AC9A5BCFF71}"/>
@@ -14972,40 +18202,40 @@
     <sortCondition ref="A2:A9"/>
   </sortState>
   <conditionalFormatting sqref="F2:F55">
-    <cfRule type="cellIs" dxfId="157" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="229" priority="8" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H55">
-    <cfRule type="cellIs" dxfId="156" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="228" priority="9" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="155" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="227" priority="10" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F55">
-    <cfRule type="cellIs" dxfId="154" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="226" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="153" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="225" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="152" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="224" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="151" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="223" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J55">
-    <cfRule type="containsText" dxfId="150" priority="5" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="222" priority="5" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="149" priority="6" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="221" priority="6" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="148" priority="7" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="220" priority="7" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15931,40 +19161,40 @@
     <sortCondition ref="A2:A4"/>
   </sortState>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="cellIs" dxfId="147" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="219" priority="8" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H53">
-    <cfRule type="cellIs" dxfId="146" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="218" priority="9" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="145" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="217" priority="10" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F53">
-    <cfRule type="cellIs" dxfId="144" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="216" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="143" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="215" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="142" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="214" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="141" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="213" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J53">
-    <cfRule type="containsText" dxfId="140" priority="5" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="212" priority="5" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="139" priority="6" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="211" priority="6" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="138" priority="7" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="210" priority="7" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17216,40 +20446,40 @@
     <sortCondition ref="A2:A23"/>
   </sortState>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="cellIs" dxfId="137" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="209" priority="12" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H53">
-    <cfRule type="cellIs" dxfId="136" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="208" priority="13" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="135" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="207" priority="14" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F53">
-    <cfRule type="cellIs" dxfId="134" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="206" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="205" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="204" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="203" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J53">
-    <cfRule type="containsText" dxfId="130" priority="9" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="202" priority="9" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="129" priority="10" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="201" priority="10" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="128" priority="11" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="200" priority="11" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17918,51 +21148,51 @@
     <mergeCell ref="F6:F10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
-    <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="199" priority="7" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H6 H11 G12:I12">
-    <cfRule type="cellIs" dxfId="126" priority="8" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="198" priority="8" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="125" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="197" priority="9" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F6 F11:F15">
-    <cfRule type="cellIs" dxfId="124" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="196" priority="10" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="195" priority="11" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="122" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="194" priority="12" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="193" priority="13" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J6">
-    <cfRule type="containsText" dxfId="120" priority="1" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="192" priority="1" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="119" priority="2" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="191" priority="2" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="118" priority="3" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="190" priority="3" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:J15">
-    <cfRule type="containsText" dxfId="117" priority="4" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="189" priority="4" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="116" priority="5" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="188" priority="5" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="115" priority="6" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="187" priority="6" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J11)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19230,40 +22460,40 @@
     <sortCondition ref="A2:A23"/>
   </sortState>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="cellIs" dxfId="114" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="186" priority="8" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H53">
-    <cfRule type="cellIs" dxfId="113" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="185" priority="9" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="184" priority="10" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F53">
-    <cfRule type="cellIs" dxfId="111" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="183" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="182" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="181" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="180" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J53">
-    <cfRule type="containsText" dxfId="107" priority="5" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="179" priority="5" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="106" priority="6" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="178" priority="6" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="105" priority="7" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="177" priority="7" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>